<commit_message>
subiendo gastos por separados en cada consorcio
</commit_message>
<xml_diff>
--- a/BELGRANO 1646/Mayo/MAYO-BLG1646.xlsx
+++ b/BELGRANO 1646/Mayo/MAYO-BLG1646.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sistema\Desktop\rc-consorcio2025\BELGRANO 1646\Mayo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FCE3E2E-B2E1-41F9-B8D4-D58C2866832E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB448BAD-8ACD-49C0-B26B-10029C718689}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,14 +19,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="1">PRORRATEO!$A$1:$N$64</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">RESUMEN!$A$1:$F$134</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">RESUMEN!$A$1:$F$143</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="169">
   <si>
     <t>consorciobelgrano1640@gmail.com</t>
   </si>
@@ -504,30 +504,9 @@
     <t>JPL - Articulos de limpieza 14/04</t>
   </si>
   <si>
-    <t>Agua porteria - Bidones - Consumo de un año</t>
-  </si>
-  <si>
-    <t>Casa ruan compra de disyuntor</t>
-  </si>
-  <si>
-    <t>Servisur - reemplazo sensor de movimiento</t>
-  </si>
-  <si>
-    <t>Casa ruan compra de sensor</t>
-  </si>
-  <si>
-    <t>Hidraulica Rubber - Cepillo pileta</t>
-  </si>
-  <si>
-    <t>Gabriel Villegas - Desvinculacion contrato ADS</t>
-  </si>
-  <si>
     <t>Fumigacion 9/04</t>
   </si>
   <si>
-    <t>Compra motor PPA - Porton acceso al montavehiculos</t>
-  </si>
-  <si>
     <t>FEUILLANT, GASTON</t>
   </si>
   <si>
@@ -549,13 +528,46 @@
     <t>Energoup MES DE MAYO</t>
   </si>
   <si>
-    <t>Mes de MAYO 23/04</t>
-  </si>
-  <si>
     <t>EN TEORIA EN ESTE PUNTO (MAYO DEL 2025) LA CAJA NOS DA BIEN, TENEMOS 1,4M EN EL BANCO Y CERCA DE 120MIL PESOS EN EFECTIVO</t>
   </si>
   <si>
     <t>Ingreso mes de ABRIL</t>
+  </si>
+  <si>
+    <t>Ruso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kromacolor  -  Recuplast </t>
+  </si>
+  <si>
+    <t>Lucas</t>
+  </si>
+  <si>
+    <t>Sur Energy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mes de MAYO </t>
+  </si>
+  <si>
+    <t>Ferreteria</t>
+  </si>
+  <si>
+    <t>Contessi provision y colocacion de 60 lts de aceite hidraulico en la sede del monta auto</t>
+  </si>
+  <si>
+    <t>Salvatierra limpieza de columna de baño desde piso 3 (inclusive) hasta el piso 10 (inclusive)</t>
+  </si>
+  <si>
+    <t>Remis Sr. Diego - Dia de paro</t>
+  </si>
+  <si>
+    <t>Alejandro 1646</t>
+  </si>
+  <si>
+    <t>Contessi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Camaras del sur 19/05 </t>
   </si>
 </sst>
 </file>
@@ -1283,7 +1295,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="244">
+  <cellXfs count="252">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
@@ -1570,92 +1582,126 @@
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="6" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="20" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="20" fillId="11" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="20" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="20" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="20" fillId="11" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="35" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="36" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="44" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1683,19 +1729,7 @@
     <xf numFmtId="0" fontId="19" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="31" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2069,7 +2103,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N144"/>
+  <dimension ref="A1:N153"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33.44140625" customWidth="1"/>
@@ -2126,10 +2160,10 @@
         <v>1</v>
       </c>
       <c r="B5" s="71" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="C5" s="71" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="D5" s="71"/>
       <c r="E5" s="72"/>
@@ -2157,26 +2191,26 @@
     <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B14" s="203" t="s">
+      <c r="B14" s="204" t="s">
         <v>135</v>
       </c>
-      <c r="C14" s="204"/>
-      <c r="D14" s="205"/>
+      <c r="C14" s="205"/>
+      <c r="D14" s="206"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B15" s="206"/>
-      <c r="C15" s="207"/>
-      <c r="D15" s="208"/>
+      <c r="B15" s="207"/>
+      <c r="C15" s="208"/>
+      <c r="D15" s="209"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="B16" s="206"/>
-      <c r="C16" s="207"/>
-      <c r="D16" s="208"/>
+      <c r="B16" s="207"/>
+      <c r="C16" s="208"/>
+      <c r="D16" s="209"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="B17" s="209"/>
-      <c r="C17" s="210"/>
-      <c r="D17" s="211"/>
+      <c r="B17" s="210"/>
+      <c r="C17" s="211"/>
+      <c r="D17" s="212"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
@@ -2201,7 +2235,7 @@
         <v>16</v>
       </c>
       <c r="B22" s="7" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="C22" s="7"/>
       <c r="D22" s="130"/>
@@ -2652,7 +2686,7 @@
         <v>140</v>
       </c>
       <c r="C53" s="7"/>
-      <c r="D53" s="199">
+      <c r="D53" s="198">
         <f>102143.27+6011.02+54099.18</f>
         <v>162253.47</v>
       </c>
@@ -2674,7 +2708,7 @@
         <v>139</v>
       </c>
       <c r="C54" s="7"/>
-      <c r="D54" s="199">
+      <c r="D54" s="198">
         <v>532295.61</v>
       </c>
       <c r="E54" s="134">
@@ -2725,169 +2759,137 @@
       <c r="F56" s="7"/>
       <c r="H56" s="150"/>
     </row>
-    <row r="57" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="195" t="s">
-        <v>141</v>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A57" s="114" t="s">
+        <v>163</v>
       </c>
       <c r="B57" s="179"/>
       <c r="C57" s="180"/>
       <c r="D57" s="200">
+        <v>700000</v>
+      </c>
+      <c r="E57" s="115"/>
+      <c r="F57" s="7"/>
+      <c r="H57" s="150"/>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A58" s="114" t="s">
+        <v>167</v>
+      </c>
+      <c r="B58" s="179"/>
+      <c r="C58" s="180"/>
+      <c r="D58" s="200">
+        <v>300000</v>
+      </c>
+      <c r="E58" s="115"/>
+      <c r="F58" s="7"/>
+      <c r="H58" s="150"/>
+    </row>
+    <row r="59" spans="1:9" ht="20.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="195" t="s">
+        <v>141</v>
+      </c>
+      <c r="B59" s="179"/>
+      <c r="C59" s="180"/>
+      <c r="D59" s="199">
         <v>330000</v>
       </c>
-      <c r="E57" s="149">
-        <f>D57</f>
+      <c r="E59" s="149">
+        <f>D59</f>
         <v>330000</v>
       </c>
-      <c r="F57" s="7"/>
-      <c r="G57" s="109">
-        <f>D57</f>
+      <c r="F59" s="7"/>
+      <c r="G59" s="109">
+        <f>D59</f>
         <v>330000</v>
       </c>
-      <c r="H57" s="161">
-        <f>E57+F57</f>
+      <c r="H59" s="161">
+        <f>E59+F59</f>
         <v>330000</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="121" t="s">
+    <row r="60" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A60" s="121" t="s">
         <v>8</v>
       </c>
-      <c r="B58" s="164"/>
-      <c r="C58" s="7"/>
-      <c r="D58" s="113">
-        <v>0</v>
-      </c>
-      <c r="E58" s="149">
-        <f t="shared" ref="E58:E63" si="8">D58*91.91%</f>
-        <v>0</v>
-      </c>
-      <c r="F58" s="134">
-        <f t="shared" ref="F58:F63" si="9">D58*8.09%</f>
-        <v>0</v>
-      </c>
-      <c r="G58" s="109">
-        <f t="shared" ref="G58:G75" si="10">D58</f>
-        <v>0</v>
-      </c>
-      <c r="H58" s="161">
-        <f t="shared" ref="H58:H75" si="11">E58+F58</f>
-        <v>0</v>
-      </c>
-      <c r="I58" t="str">
-        <f t="shared" ref="I58:I74" si="12">IF(G58=H58, "", "Error")</f>
+      <c r="B60" s="164"/>
+      <c r="C60" s="7"/>
+      <c r="D60" s="198">
+        <v>118708.63</v>
+      </c>
+      <c r="E60" s="149">
+        <f t="shared" ref="E60:E65" si="8">D60*91.91%</f>
+        <v>109105.10183299999</v>
+      </c>
+      <c r="F60" s="134">
+        <f t="shared" ref="F60:F65" si="9">D60*8.09%</f>
+        <v>9603.5281670000004</v>
+      </c>
+      <c r="G60" s="109">
+        <f t="shared" ref="G60:G84" si="10">D60</f>
+        <v>118708.63</v>
+      </c>
+      <c r="H60" s="161">
+        <f t="shared" ref="H60:H84" si="11">E60+F60</f>
+        <v>118708.62999999999</v>
+      </c>
+      <c r="I60" t="str">
+        <f t="shared" ref="I60:I83" si="12">IF(G60=H60, "", "Error")</f>
         <v/>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" s="94" t="s">
-        <v>161</v>
-      </c>
-      <c r="B59" s="7"/>
-      <c r="C59" s="7"/>
-      <c r="D59" s="113">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A61" s="94" t="s">
+        <v>154</v>
+      </c>
+      <c r="B61" s="7"/>
+      <c r="C61" s="7"/>
+      <c r="D61" s="198">
         <v>129675</v>
       </c>
-      <c r="E59" s="149">
+      <c r="E61" s="149">
         <f t="shared" si="8"/>
         <v>119184.2925</v>
       </c>
-      <c r="F59" s="134">
+      <c r="F61" s="134">
         <f t="shared" si="9"/>
         <v>10490.7075</v>
       </c>
-      <c r="G59" s="109">
+      <c r="G61" s="109">
         <f t="shared" si="10"/>
         <v>129675</v>
       </c>
-      <c r="H59" s="161">
+      <c r="H61" s="161">
         <f t="shared" si="11"/>
         <v>129675</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" s="94" t="s">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A62" s="94" t="s">
         <v>9</v>
       </c>
-      <c r="B60" s="7" t="s">
+      <c r="B62" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="C60" s="7"/>
-      <c r="D60" s="113">
+      <c r="C62" s="7"/>
+      <c r="D62" s="113">
         <v>74622</v>
       </c>
-      <c r="E60" s="149">
+      <c r="E62" s="149">
         <f t="shared" si="8"/>
         <v>68585.080199999997</v>
       </c>
-      <c r="F60" s="134">
+      <c r="F62" s="134">
         <f t="shared" si="9"/>
         <v>6036.9197999999997</v>
       </c>
-      <c r="G60" s="109">
+      <c r="G62" s="109">
         <f t="shared" si="10"/>
         <v>74622</v>
       </c>
-      <c r="H60" s="161">
+      <c r="H62" s="161">
         <f t="shared" si="11"/>
         <v>74622</v>
-      </c>
-      <c r="I60" t="str">
-        <f t="shared" si="12"/>
-        <v/>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" s="94" t="s">
-        <v>11</v>
-      </c>
-      <c r="B61" s="7" t="s">
-        <v>143</v>
-      </c>
-      <c r="C61" s="7"/>
-      <c r="D61" s="113">
-        <f>314851+309690.68</f>
-        <v>624541.67999999993</v>
-      </c>
-      <c r="E61" s="149">
-        <f t="shared" si="8"/>
-        <v>574016.25808799989</v>
-      </c>
-      <c r="F61" s="134">
-        <f t="shared" si="9"/>
-        <v>50525.421911999998</v>
-      </c>
-      <c r="G61" s="109">
-        <f t="shared" si="10"/>
-        <v>624541.67999999993</v>
-      </c>
-      <c r="H61" s="161"/>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A62" s="129" t="s">
-        <v>10</v>
-      </c>
-      <c r="B62" s="98" t="s">
-        <v>142</v>
-      </c>
-      <c r="C62" s="98"/>
-      <c r="D62" s="113">
-        <v>909879.28</v>
-      </c>
-      <c r="E62" s="149">
-        <f t="shared" si="8"/>
-        <v>836270.046248</v>
-      </c>
-      <c r="F62" s="134">
-        <f t="shared" si="9"/>
-        <v>73609.233752</v>
-      </c>
-      <c r="G62" s="109">
-        <f t="shared" si="10"/>
-        <v>909879.28</v>
-      </c>
-      <c r="H62" s="161">
-        <f t="shared" si="11"/>
-        <v>909879.28</v>
       </c>
       <c r="I62" t="str">
         <f t="shared" si="12"/>
@@ -2895,1062 +2897,1240 @@
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A63" s="129" t="s">
-        <v>145</v>
-      </c>
-      <c r="B63" s="98"/>
-      <c r="C63" s="98"/>
+      <c r="A63" s="94" t="s">
+        <v>11</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="C63" s="7"/>
       <c r="D63" s="113">
-        <v>40000</v>
+        <f>314851+309690.68</f>
+        <v>624541.67999999993</v>
       </c>
       <c r="E63" s="149">
         <f t="shared" si="8"/>
-        <v>36764</v>
+        <v>574016.25808799989</v>
       </c>
       <c r="F63" s="134">
         <f t="shared" si="9"/>
-        <v>3236</v>
+        <v>50525.421911999998</v>
       </c>
       <c r="G63" s="109">
         <f t="shared" si="10"/>
+        <v>624541.67999999993</v>
+      </c>
+      <c r="H63" s="161"/>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A64" s="129" t="s">
+        <v>10</v>
+      </c>
+      <c r="B64" s="98" t="s">
+        <v>142</v>
+      </c>
+      <c r="C64" s="98"/>
+      <c r="D64" s="198">
+        <v>909788.31</v>
+      </c>
+      <c r="E64" s="149">
+        <f t="shared" si="8"/>
+        <v>836186.43572099996</v>
+      </c>
+      <c r="F64" s="134">
+        <f t="shared" si="9"/>
+        <v>73601.874279000011</v>
+      </c>
+      <c r="G64" s="109">
+        <f t="shared" si="10"/>
+        <v>909788.31</v>
+      </c>
+      <c r="H64" s="161">
+        <f t="shared" si="11"/>
+        <v>909788.30999999994</v>
+      </c>
+      <c r="I64" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A65" s="129" t="s">
+        <v>145</v>
+      </c>
+      <c r="B65" s="98"/>
+      <c r="C65" s="98"/>
+      <c r="D65" s="113">
         <v>40000</v>
       </c>
-      <c r="H63" s="161">
+      <c r="E65" s="149">
+        <f t="shared" si="8"/>
+        <v>36764</v>
+      </c>
+      <c r="F65" s="134">
+        <f t="shared" si="9"/>
+        <v>3236</v>
+      </c>
+      <c r="G65" s="109">
+        <f t="shared" si="10"/>
+        <v>40000</v>
+      </c>
+      <c r="H65" s="161">
         <f t="shared" si="11"/>
         <v>40000</v>
       </c>
-      <c r="I63" t="str">
+      <c r="I65" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A64" s="98" t="s">
-        <v>148</v>
-      </c>
-      <c r="B64" s="183"/>
-      <c r="C64" s="184"/>
-      <c r="D64" s="113">
-        <v>113500</v>
-      </c>
-      <c r="E64" s="149">
-        <f t="shared" ref="E64:E69" si="13">D64</f>
-        <v>113500</v>
-      </c>
-      <c r="F64" s="134"/>
-      <c r="G64" s="109">
-        <f t="shared" si="10"/>
-        <v>113500</v>
-      </c>
-      <c r="H64" s="161">
-        <f t="shared" si="11"/>
-        <v>113500</v>
-      </c>
-      <c r="I64" s="181"/>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A65" s="215" t="s">
-        <v>150</v>
-      </c>
-      <c r="B65" s="216"/>
-      <c r="C65" s="217"/>
-      <c r="D65" s="113">
-        <v>22000</v>
-      </c>
-      <c r="E65" s="149">
-        <f t="shared" si="13"/>
-        <v>22000</v>
-      </c>
-      <c r="F65" s="134"/>
-      <c r="G65" s="109">
-        <f t="shared" si="10"/>
-        <v>22000</v>
-      </c>
-      <c r="H65" s="161">
-        <f t="shared" si="11"/>
-        <v>22000</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="215" t="s">
-        <v>149</v>
-      </c>
-      <c r="B66" s="216"/>
-      <c r="C66" s="217"/>
-      <c r="D66" s="113">
-        <v>25000</v>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A66" s="98" t="s">
+        <v>168</v>
+      </c>
+      <c r="B66" s="183"/>
+      <c r="C66" s="184"/>
+      <c r="D66" s="198">
+        <v>235500</v>
       </c>
       <c r="E66" s="149">
-        <f t="shared" si="13"/>
-        <v>25000</v>
+        <f t="shared" ref="E66:E78" si="13">D66</f>
+        <v>235500</v>
       </c>
       <c r="F66" s="134"/>
       <c r="G66" s="109">
-        <f>D66</f>
-        <v>25000</v>
+        <f t="shared" si="10"/>
+        <v>235500</v>
       </c>
       <c r="H66" s="161">
         <f t="shared" si="11"/>
-        <v>25000</v>
-      </c>
-      <c r="I66" t="str">
-        <f>IF(G66=H66, "", "Error")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="215" t="s">
+        <v>235500</v>
+      </c>
+      <c r="I66" s="181"/>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A67" s="216" t="s">
         <v>157</v>
       </c>
-      <c r="B67" s="216"/>
-      <c r="C67" s="217"/>
-      <c r="D67" s="199">
-        <v>6000</v>
+      <c r="B67" s="217"/>
+      <c r="C67" s="218"/>
+      <c r="D67" s="198">
+        <v>111026</v>
       </c>
       <c r="E67" s="149">
         <f t="shared" si="13"/>
-        <v>6000</v>
+        <v>111026</v>
       </c>
       <c r="F67" s="134"/>
       <c r="G67" s="109">
-        <f>D67</f>
-        <v>6000</v>
+        <f t="shared" si="10"/>
+        <v>111026</v>
       </c>
       <c r="H67" s="161">
         <f t="shared" si="11"/>
-        <v>6000</v>
+        <v>111026</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="198" t="s">
-        <v>152</v>
-      </c>
-      <c r="B68" s="193"/>
-      <c r="C68" s="194"/>
-      <c r="D68" s="113">
-        <v>200000</v>
+      <c r="A68" s="216" t="s">
+        <v>160</v>
+      </c>
+      <c r="B68" s="217"/>
+      <c r="C68" s="218"/>
+      <c r="D68" s="198">
+        <f>104002.96</f>
+        <v>104002.96</v>
       </c>
       <c r="E68" s="149">
         <f t="shared" si="13"/>
-        <v>200000</v>
+        <v>104002.96</v>
       </c>
       <c r="F68" s="134"/>
       <c r="G68" s="109">
         <f>D68</f>
-        <v>200000</v>
+        <v>104002.96</v>
       </c>
       <c r="H68" s="161">
         <f t="shared" si="11"/>
-        <v>200000</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A69" s="215" t="s">
-        <v>153</v>
-      </c>
-      <c r="B69" s="216"/>
-      <c r="C69" s="217"/>
-      <c r="D69" s="199">
-        <v>66000</v>
+        <v>104002.96</v>
+      </c>
+      <c r="I68" t="str">
+        <f>IF(G68=H68, "", "Error")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="216" t="s">
+        <v>160</v>
+      </c>
+      <c r="B69" s="217"/>
+      <c r="C69" s="218"/>
+      <c r="D69" s="198">
+        <f>104002.96</f>
+        <v>104002.96</v>
       </c>
       <c r="E69" s="149">
         <f t="shared" si="13"/>
+        <v>104002.96</v>
+      </c>
+      <c r="F69" s="134"/>
+      <c r="G69" s="109"/>
+      <c r="H69" s="161"/>
+    </row>
+    <row r="70" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="216" t="s">
+        <v>160</v>
+      </c>
+      <c r="B70" s="217"/>
+      <c r="C70" s="218"/>
+      <c r="D70" s="198">
+        <f>104002.96</f>
+        <v>104002.96</v>
+      </c>
+      <c r="E70" s="149">
+        <f t="shared" si="13"/>
+        <v>104002.96</v>
+      </c>
+      <c r="F70" s="134"/>
+      <c r="G70" s="109"/>
+      <c r="H70" s="161"/>
+    </row>
+    <row r="71" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A71" s="216" t="s">
+        <v>160</v>
+      </c>
+      <c r="B71" s="217"/>
+      <c r="C71" s="218"/>
+      <c r="D71" s="198">
+        <f>104002.96</f>
+        <v>104002.96</v>
+      </c>
+      <c r="E71" s="149">
+        <f t="shared" si="13"/>
+        <v>104002.96</v>
+      </c>
+      <c r="F71" s="134"/>
+      <c r="G71" s="109"/>
+      <c r="H71" s="161"/>
+    </row>
+    <row r="72" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A72" s="201" t="s">
+        <v>166</v>
+      </c>
+      <c r="B72" s="175"/>
+      <c r="C72" s="202"/>
+      <c r="D72" s="198">
+        <v>100419.01</v>
+      </c>
+      <c r="E72" s="149"/>
+      <c r="F72" s="134"/>
+      <c r="G72" s="109"/>
+      <c r="H72" s="161"/>
+    </row>
+    <row r="73" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A73" s="201" t="s">
+        <v>166</v>
+      </c>
+      <c r="B73" s="175"/>
+      <c r="C73" s="202"/>
+      <c r="D73" s="198">
+        <v>97003.05</v>
+      </c>
+      <c r="E73" s="149"/>
+      <c r="F73" s="134"/>
+      <c r="G73" s="109"/>
+      <c r="H73" s="161"/>
+    </row>
+    <row r="74" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A74" s="227" t="s">
+        <v>150</v>
+      </c>
+      <c r="B74" s="228"/>
+      <c r="C74" s="229"/>
+      <c r="D74" s="198">
+        <v>6000</v>
+      </c>
+      <c r="E74" s="149">
+        <f t="shared" si="13"/>
+        <v>6000</v>
+      </c>
+      <c r="F74" s="134"/>
+      <c r="G74" s="109">
+        <f>D74</f>
+        <v>6000</v>
+      </c>
+      <c r="H74" s="161">
+        <f t="shared" si="11"/>
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A75" s="227" t="s">
+        <v>165</v>
+      </c>
+      <c r="B75" s="228"/>
+      <c r="C75" s="229"/>
+      <c r="D75" s="198">
+        <v>7000</v>
+      </c>
+      <c r="E75" s="149">
+        <f t="shared" si="13"/>
+        <v>7000</v>
+      </c>
+      <c r="F75" s="134"/>
+      <c r="G75" s="109"/>
+      <c r="H75" s="161"/>
+    </row>
+    <row r="76" spans="1:9" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A76" s="203"/>
+      <c r="B76" s="193"/>
+      <c r="C76" s="194"/>
+      <c r="D76" s="198">
+        <v>98393.96</v>
+      </c>
+      <c r="E76" s="149">
+        <f t="shared" si="13"/>
+        <v>98393.96</v>
+      </c>
+      <c r="F76" s="134"/>
+      <c r="G76" s="109">
+        <f>D76</f>
+        <v>98393.96</v>
+      </c>
+      <c r="H76" s="161">
+        <f t="shared" si="11"/>
+        <v>98393.96</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A77" s="227" t="s">
+        <v>147</v>
+      </c>
+      <c r="B77" s="228"/>
+      <c r="C77" s="229"/>
+      <c r="D77" s="198">
         <v>66000</v>
       </c>
-      <c r="F69" s="134"/>
-      <c r="G69" s="109">
+      <c r="E77" s="149">
+        <f t="shared" si="13"/>
+        <v>66000</v>
+      </c>
+      <c r="F77" s="134"/>
+      <c r="G77" s="109">
         <f t="shared" si="10"/>
         <v>66000</v>
       </c>
-      <c r="H69" s="161">
+      <c r="H77" s="161">
         <f t="shared" si="11"/>
         <v>66000</v>
       </c>
-      <c r="I69" t="str">
+      <c r="I77" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
     </row>
-    <row r="70" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="7" t="s">
+    <row r="78" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A78" s="230" t="s">
+        <v>164</v>
+      </c>
+      <c r="B78" s="231"/>
+      <c r="C78" s="194"/>
+      <c r="D78" s="198">
+        <v>218400</v>
+      </c>
+      <c r="E78" s="149">
+        <f t="shared" si="13"/>
+        <v>218400</v>
+      </c>
+      <c r="F78" s="134"/>
+      <c r="G78" s="109"/>
+      <c r="H78" s="161"/>
+    </row>
+    <row r="79" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A79" s="7" t="s">
         <v>120</v>
       </c>
-      <c r="B70" s="7" t="s">
-        <v>162</v>
-      </c>
-      <c r="C70" s="7"/>
-      <c r="D70" s="113">
+      <c r="B79" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="C79" s="7"/>
+      <c r="D79" s="198">
         <v>79895</v>
       </c>
-      <c r="E70" s="149">
-        <f t="shared" ref="E70:E75" si="14">D70</f>
+      <c r="E79" s="149">
+        <f t="shared" ref="E79:E84" si="14">D79</f>
         <v>79895</v>
       </c>
-      <c r="F70" s="7"/>
-      <c r="G70" s="109">
+      <c r="F79" s="7"/>
+      <c r="G79" s="109">
         <f t="shared" si="10"/>
         <v>79895</v>
       </c>
-      <c r="H70" s="161">
+      <c r="H79" s="161">
         <f t="shared" si="11"/>
         <v>79895</v>
       </c>
-      <c r="I70" t="str">
+      <c r="I79" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
     </row>
-    <row r="71" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="94" t="s">
-        <v>147</v>
-      </c>
-      <c r="B71" s="7"/>
-      <c r="C71" s="7"/>
-      <c r="D71" s="113">
-        <v>96300</v>
-      </c>
-      <c r="E71" s="149">
-        <f t="shared" ref="E71" si="15">D71*91.91%</f>
-        <v>88509.329999999987</v>
-      </c>
-      <c r="F71" s="134">
-        <f t="shared" ref="F71" si="16">D71*8.09%</f>
-        <v>7790.67</v>
-      </c>
-      <c r="G71" s="109">
+    <row r="80" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A80" s="94" t="s">
+        <v>162</v>
+      </c>
+      <c r="B80" s="7"/>
+      <c r="C80" s="7"/>
+      <c r="D80" s="198">
+        <v>6530.7</v>
+      </c>
+      <c r="E80" s="149">
+        <f t="shared" ref="E80" si="15">D80*91.91%</f>
+        <v>6002.3663699999997</v>
+      </c>
+      <c r="F80" s="134">
+        <f t="shared" ref="F80" si="16">D80*8.09%</f>
+        <v>528.33362999999997</v>
+      </c>
+      <c r="G80" s="109">
         <f t="shared" si="10"/>
-        <v>96300</v>
-      </c>
-      <c r="H71" s="161">
+        <v>6530.7</v>
+      </c>
+      <c r="H80" s="161">
         <f t="shared" si="11"/>
-        <v>96299.999999999985</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="7" t="s">
-        <v>154</v>
-      </c>
-      <c r="B72" s="7"/>
-      <c r="C72" s="7"/>
-      <c r="D72" s="113">
-        <v>460000</v>
-      </c>
-      <c r="E72" s="149">
+        <v>6530.7</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A81" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B81" s="7"/>
+      <c r="C81" s="7"/>
+      <c r="D81" s="198">
+        <v>10391.24</v>
+      </c>
+      <c r="E81" s="149">
         <f t="shared" si="14"/>
-        <v>460000</v>
-      </c>
-      <c r="F72" s="7"/>
-      <c r="G72" s="109">
+        <v>10391.24</v>
+      </c>
+      <c r="F81" s="7"/>
+      <c r="G81" s="109">
         <f t="shared" si="10"/>
-        <v>460000</v>
-      </c>
-      <c r="H72" s="161"/>
-    </row>
-    <row r="73" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="7" t="s">
-        <v>156</v>
-      </c>
-      <c r="B73" s="7"/>
-      <c r="C73" s="7"/>
-      <c r="D73" s="199">
+        <v>10391.24</v>
+      </c>
+      <c r="H81" s="161"/>
+    </row>
+    <row r="82" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A82" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B82" s="7"/>
+      <c r="C82" s="7"/>
+      <c r="D82" s="198">
         <v>120000</v>
       </c>
-      <c r="E73" s="149">
+      <c r="E82" s="149">
         <f t="shared" si="14"/>
         <v>120000</v>
       </c>
-      <c r="F73" s="7"/>
-      <c r="G73" s="109">
+      <c r="F82" s="7"/>
+      <c r="G82" s="109">
         <f t="shared" si="10"/>
         <v>120000</v>
       </c>
-      <c r="H73" s="161"/>
-    </row>
-    <row r="74" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="98" t="s">
-        <v>151</v>
-      </c>
-      <c r="B74" s="114"/>
-      <c r="C74" s="163"/>
-      <c r="D74" s="113">
-        <v>11800</v>
-      </c>
-      <c r="E74" s="149">
+      <c r="H82" s="161"/>
+    </row>
+    <row r="83" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A83" s="98" t="s">
+        <v>159</v>
+      </c>
+      <c r="B83" s="114"/>
+      <c r="C83" s="163"/>
+      <c r="D83" s="198">
+        <v>80000</v>
+      </c>
+      <c r="E83" s="149">
         <f t="shared" si="14"/>
-        <v>11800</v>
-      </c>
-      <c r="F74" s="134"/>
-      <c r="G74" s="109">
+        <v>80000</v>
+      </c>
+      <c r="F83" s="134"/>
+      <c r="G83" s="109">
         <f t="shared" si="10"/>
-        <v>11800</v>
-      </c>
-      <c r="H74" s="161">
+        <v>80000</v>
+      </c>
+      <c r="H83" s="161">
         <f t="shared" si="11"/>
-        <v>11800</v>
-      </c>
-      <c r="I74" t="str">
+        <v>80000</v>
+      </c>
+      <c r="I83" t="str">
         <f t="shared" si="12"/>
         <v/>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A75" s="155"/>
-      <c r="B75" s="156"/>
-      <c r="C75" s="156"/>
-      <c r="D75" s="167"/>
-      <c r="E75" s="149">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A84" s="155"/>
+      <c r="B84" s="156"/>
+      <c r="C84" s="156"/>
+      <c r="D84" s="167"/>
+      <c r="E84" s="149">
         <f t="shared" si="14"/>
         <v>0</v>
       </c>
-      <c r="F75" s="134"/>
-      <c r="G75" s="109">
+      <c r="F84" s="134"/>
+      <c r="G84" s="109">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="H75" s="161">
+      <c r="H84" s="161">
         <f t="shared" si="11"/>
         <v>0</v>
       </c>
-      <c r="I75" t="str">
-        <f>IF(G75=H75, "", "Error")</f>
+      <c r="I84" t="str">
+        <f>IF(G84=H84, "", "Error")</f>
         <v/>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A76" s="96" t="s">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A85" s="96" t="s">
         <v>12</v>
       </c>
-      <c r="B76" s="96"/>
-      <c r="C76" s="96"/>
-      <c r="D76" s="108">
-        <f>SUM(D58:D75)</f>
-        <v>2979212.96</v>
-      </c>
-      <c r="E76" s="108">
-        <f>SUM(E58:E75)</f>
-        <v>2827524.007036</v>
-      </c>
-      <c r="F76" s="108">
-        <f>SUM(F58:F75)</f>
-        <v>151688.95296400003</v>
-      </c>
-      <c r="G76" s="109">
-        <f>E76+F76</f>
-        <v>2979212.96</v>
-      </c>
-      <c r="H76" s="150" t="str">
-        <f>IF(D76=G76, "", "Error")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="77" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="7"/>
-      <c r="B77" s="7"/>
-      <c r="C77" s="7"/>
-      <c r="D77" s="189"/>
-      <c r="E77" s="115"/>
-      <c r="F77" s="7"/>
-      <c r="H77" s="150"/>
-    </row>
-    <row r="78" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="7"/>
-      <c r="B78" s="7"/>
-      <c r="C78" s="7"/>
-      <c r="D78" s="189"/>
-      <c r="E78" s="114"/>
-      <c r="F78" s="7"/>
-      <c r="H78" s="150"/>
-    </row>
-    <row r="79" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="7"/>
-      <c r="B79" s="7"/>
-      <c r="C79" s="7"/>
-      <c r="D79" s="189"/>
-      <c r="E79" s="114"/>
-      <c r="F79" s="7"/>
-      <c r="H79" s="150"/>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A80" s="94" t="s">
-        <v>146</v>
-      </c>
-      <c r="B80" s="98"/>
-      <c r="C80" s="7"/>
-      <c r="D80" s="113">
-        <v>186900</v>
-      </c>
-      <c r="E80" s="149">
-        <f>D80*91.91%</f>
-        <v>171779.78999999998</v>
-      </c>
-      <c r="F80" s="134">
-        <f>D80*8.09%</f>
-        <v>15120.21</v>
-      </c>
-      <c r="G80" s="160"/>
-      <c r="H80" s="150"/>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A81" s="98"/>
-      <c r="B81" s="162"/>
-      <c r="C81" s="7"/>
-      <c r="D81" s="113"/>
-      <c r="E81" s="149">
-        <f>D81</f>
-        <v>0</v>
-      </c>
-      <c r="F81" s="134"/>
-      <c r="H81" s="150"/>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A82" s="7"/>
-      <c r="B82" s="7"/>
-      <c r="C82" s="7"/>
-      <c r="D82" s="113"/>
-      <c r="E82" s="165">
-        <f>D82</f>
-        <v>0</v>
-      </c>
-      <c r="F82" s="7"/>
-      <c r="H82" s="150"/>
-      <c r="I82" s="109"/>
-    </row>
-    <row r="83" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="95" t="s">
-        <v>17</v>
-      </c>
-      <c r="B83" s="95"/>
-      <c r="C83" s="95"/>
-      <c r="D83" s="107">
-        <f>SUM(D80:D82)</f>
-        <v>186900</v>
-      </c>
-      <c r="E83" s="107">
-        <f>SUM(E80:E82)</f>
-        <v>171779.78999999998</v>
-      </c>
-      <c r="F83" s="107">
-        <f>SUM(F80:F82)</f>
-        <v>15120.21</v>
-      </c>
-      <c r="G83" s="109">
-        <f>E83+F83</f>
-        <v>186899.99999999997</v>
-      </c>
-      <c r="H83" s="150" t="str">
-        <f>IF(D83=G83, "", "Error")</f>
-        <v/>
-      </c>
-      <c r="J83" s="109"/>
-    </row>
-    <row r="84" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="7"/>
-      <c r="B84" s="7"/>
-      <c r="C84" s="7"/>
-      <c r="D84" s="189"/>
-      <c r="E84" s="115"/>
-      <c r="F84" s="7"/>
-      <c r="H84" s="150"/>
-    </row>
-    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="7"/>
-      <c r="B85" s="7"/>
-      <c r="C85" s="7"/>
-      <c r="D85" s="189"/>
-      <c r="E85" s="114"/>
-      <c r="F85" s="7"/>
-      <c r="H85" s="150"/>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A86" s="94" t="s">
-        <v>13</v>
-      </c>
+      <c r="B85" s="96"/>
+      <c r="C85" s="96"/>
+      <c r="D85" s="108">
+        <f>SUM(D60:D84)</f>
+        <v>3549906.42</v>
+      </c>
+      <c r="E85" s="108">
+        <f>SUM(E60:E84)</f>
+        <v>3198461.5747119999</v>
+      </c>
+      <c r="F85" s="108">
+        <f>SUM(F60:F84)</f>
+        <v>154022.78528800001</v>
+      </c>
+      <c r="G85" s="109">
+        <f>E85+F85</f>
+        <v>3352484.36</v>
+      </c>
+      <c r="H85" s="150" t="str">
+        <f>IF(D85=G85, "", "Error")</f>
+        <v>Error</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A86" s="7"/>
       <c r="B86" s="7"/>
       <c r="C86" s="7"/>
       <c r="D86" s="189"/>
-      <c r="E86" s="114"/>
+      <c r="E86" s="115"/>
       <c r="F86" s="7"/>
       <c r="H86" s="150"/>
     </row>
-    <row r="87" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="94" t="s">
-        <v>14</v>
-      </c>
-      <c r="B87" s="7" t="s">
-        <v>117</v>
-      </c>
+    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A87" s="7"/>
+      <c r="B87" s="7"/>
       <c r="C87" s="7"/>
-      <c r="D87" s="199">
-        <v>222264.92</v>
-      </c>
-      <c r="E87" s="149">
-        <f>D87*91.91%</f>
-        <v>204283.68797199999</v>
-      </c>
-      <c r="F87" s="134">
-        <f>D87*8.09%</f>
-        <v>17981.232028000002</v>
-      </c>
+      <c r="D87" s="189"/>
+      <c r="E87" s="114"/>
+      <c r="F87" s="7"/>
       <c r="H87" s="150"/>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A88" s="94" t="s">
-        <v>108</v>
-      </c>
+    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A88" s="7"/>
       <c r="B88" s="7"/>
       <c r="C88" s="7"/>
-      <c r="D88" s="199">
-        <v>28000</v>
-      </c>
-      <c r="E88" s="149">
-        <f>D88*91.91%</f>
-        <v>25734.799999999999</v>
-      </c>
-      <c r="F88" s="134">
-        <f>D88*8.09%</f>
-        <v>2265.1999999999998</v>
-      </c>
+      <c r="D88" s="189"/>
+      <c r="E88" s="114"/>
+      <c r="F88" s="7"/>
       <c r="H88" s="150"/>
-      <c r="J88" s="113"/>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A89" s="7"/>
-      <c r="B89" s="7"/>
+      <c r="A89" s="94" t="s">
+        <v>146</v>
+      </c>
+      <c r="B89" s="98"/>
       <c r="C89" s="7"/>
-      <c r="D89" s="189"/>
-      <c r="E89" s="116"/>
-      <c r="F89" s="7"/>
+      <c r="D89" s="113">
+        <v>186900</v>
+      </c>
+      <c r="E89" s="149">
+        <f>D89*91.91%</f>
+        <v>171779.78999999998</v>
+      </c>
+      <c r="F89" s="134">
+        <f>D89*8.09%</f>
+        <v>15120.21</v>
+      </c>
+      <c r="G89" s="160"/>
       <c r="H89" s="150"/>
-      <c r="J89" s="109"/>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A90" s="95" t="s">
-        <v>101</v>
-      </c>
-      <c r="B90" s="95"/>
-      <c r="C90" s="95"/>
-      <c r="D90" s="107">
-        <f>SUM(D87:D89)</f>
-        <v>250264.92</v>
-      </c>
-      <c r="E90" s="107">
-        <f>SUM(E87:E89)</f>
-        <v>230018.48797199997</v>
-      </c>
-      <c r="F90" s="107">
-        <f>SUM(F87:F89)</f>
-        <v>20246.432028000003</v>
-      </c>
-      <c r="G90" s="109">
-        <f>E90+F90</f>
-        <v>250264.91999999998</v>
-      </c>
-      <c r="H90" s="150" t="str">
-        <f>IF(D90=G90, "", "Error")</f>
-        <v/>
-      </c>
-      <c r="J90" s="109"/>
-    </row>
-    <row r="91" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A90" s="98"/>
+      <c r="B90" s="162"/>
+      <c r="C90" s="7"/>
+      <c r="D90" s="113"/>
+      <c r="E90" s="149">
+        <f>D90</f>
+        <v>0</v>
+      </c>
+      <c r="F90" s="134"/>
+      <c r="H90" s="150"/>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" s="7"/>
       <c r="B91" s="7"/>
       <c r="C91" s="7"/>
       <c r="D91" s="113"/>
-      <c r="E91" s="117"/>
+      <c r="E91" s="165">
+        <f>D91</f>
+        <v>0</v>
+      </c>
       <c r="F91" s="7"/>
       <c r="H91" s="150"/>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A92" s="94" t="s">
+      <c r="I91" s="109"/>
+    </row>
+    <row r="92" spans="1:10" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A92" s="95" t="s">
+        <v>17</v>
+      </c>
+      <c r="B92" s="95"/>
+      <c r="C92" s="95"/>
+      <c r="D92" s="107">
+        <f>SUM(D89:D91)</f>
+        <v>186900</v>
+      </c>
+      <c r="E92" s="107">
+        <f>SUM(E89:E91)</f>
+        <v>171779.78999999998</v>
+      </c>
+      <c r="F92" s="107">
+        <f>SUM(F89:F91)</f>
+        <v>15120.21</v>
+      </c>
+      <c r="G92" s="109">
+        <f>E92+F92</f>
+        <v>186899.99999999997</v>
+      </c>
+      <c r="H92" s="150" t="str">
+        <f>IF(D92=G92, "", "Error")</f>
+        <v/>
+      </c>
+      <c r="J92" s="109"/>
+    </row>
+    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A93" s="7"/>
+      <c r="B93" s="7"/>
+      <c r="C93" s="7"/>
+      <c r="D93" s="189"/>
+      <c r="E93" s="115"/>
+      <c r="F93" s="7"/>
+      <c r="H93" s="150"/>
+    </row>
+    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A94" s="7"/>
+      <c r="B94" s="7"/>
+      <c r="C94" s="7"/>
+      <c r="D94" s="189"/>
+      <c r="E94" s="114"/>
+      <c r="F94" s="7"/>
+      <c r="H94" s="150"/>
+    </row>
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A95" s="94" t="s">
+        <v>13</v>
+      </c>
+      <c r="B95" s="7"/>
+      <c r="C95" s="7"/>
+      <c r="D95" s="189"/>
+      <c r="E95" s="114"/>
+      <c r="F95" s="7"/>
+      <c r="H95" s="150"/>
+    </row>
+    <row r="96" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A96" s="94" t="s">
+        <v>14</v>
+      </c>
+      <c r="B96" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="C96" s="7"/>
+      <c r="D96" s="198">
+        <v>222264.92</v>
+      </c>
+      <c r="E96" s="149">
+        <f>D96*91.91%</f>
+        <v>204283.68797199999</v>
+      </c>
+      <c r="F96" s="134">
+        <f>D96*8.09%</f>
+        <v>17981.232028000002</v>
+      </c>
+      <c r="H96" s="150"/>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A97" s="94" t="s">
+        <v>108</v>
+      </c>
+      <c r="B97" s="7"/>
+      <c r="C97" s="7"/>
+      <c r="D97" s="198">
+        <v>28000</v>
+      </c>
+      <c r="E97" s="149">
+        <f>D97*91.91%</f>
+        <v>25734.799999999999</v>
+      </c>
+      <c r="F97" s="134">
+        <f>D97*8.09%</f>
+        <v>2265.1999999999998</v>
+      </c>
+      <c r="H97" s="150"/>
+      <c r="J97" s="113"/>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A98" s="7"/>
+      <c r="B98" s="7"/>
+      <c r="C98" s="7"/>
+      <c r="D98" s="189"/>
+      <c r="E98" s="116"/>
+      <c r="F98" s="7"/>
+      <c r="H98" s="150"/>
+      <c r="J98" s="109"/>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A99" s="95" t="s">
+        <v>101</v>
+      </c>
+      <c r="B99" s="95"/>
+      <c r="C99" s="95"/>
+      <c r="D99" s="107">
+        <f>SUM(D96:D98)</f>
+        <v>250264.92</v>
+      </c>
+      <c r="E99" s="107">
+        <f>SUM(E96:E98)</f>
+        <v>230018.48797199997</v>
+      </c>
+      <c r="F99" s="107">
+        <f>SUM(F96:F98)</f>
+        <v>20246.432028000003</v>
+      </c>
+      <c r="G99" s="109">
+        <f>E99+F99</f>
+        <v>250264.91999999998</v>
+      </c>
+      <c r="H99" s="150" t="str">
+        <f>IF(D99=G99, "", "Error")</f>
+        <v/>
+      </c>
+      <c r="J99" s="109"/>
+    </row>
+    <row r="100" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A100" s="7"/>
+      <c r="B100" s="7"/>
+      <c r="C100" s="7"/>
+      <c r="D100" s="113"/>
+      <c r="E100" s="117"/>
+      <c r="F100" s="7"/>
+      <c r="H100" s="150"/>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A101" s="94" t="s">
         <v>102</v>
       </c>
-      <c r="B92" s="7"/>
-      <c r="C92" s="7"/>
-      <c r="D92" s="113">
+      <c r="B101" s="7"/>
+      <c r="C101" s="7"/>
+      <c r="D101" s="113">
         <v>96626.92</v>
       </c>
-      <c r="E92" s="149">
-        <f>D92*91.91%</f>
+      <c r="E101" s="149">
+        <f>D101*91.91%</f>
         <v>88809.802171999996</v>
       </c>
-      <c r="F92" s="134">
-        <f>D92*8.09%</f>
+      <c r="F101" s="134">
+        <f>D101*8.09%</f>
         <v>7817.1178279999995</v>
       </c>
-      <c r="H92" s="150"/>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A93" s="94" t="s">
+      <c r="H101" s="150"/>
+    </row>
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A102" s="94" t="s">
         <v>103</v>
       </c>
-      <c r="B93" s="7"/>
-      <c r="C93" s="122"/>
-      <c r="D93" s="113">
+      <c r="B102" s="7"/>
+      <c r="C102" s="122"/>
+      <c r="D102" s="113">
         <v>44400</v>
       </c>
-      <c r="E93" s="149">
-        <f>D93*91.91%</f>
+      <c r="E102" s="149">
+        <f>D102*91.91%</f>
         <v>40808.039999999994</v>
       </c>
-      <c r="F93" s="134">
-        <f>D93*8.09%</f>
+      <c r="F102" s="134">
+        <f>D102*8.09%</f>
         <v>3591.96</v>
       </c>
-      <c r="H93" s="150"/>
-    </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A94" s="95" t="s">
+      <c r="H102" s="150"/>
+    </row>
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A103" s="95" t="s">
         <v>15</v>
       </c>
-      <c r="B94" s="95"/>
-      <c r="C94" s="95"/>
-      <c r="D94" s="158">
-        <f>SUM(D92:D93)</f>
+      <c r="B103" s="95"/>
+      <c r="C103" s="95"/>
+      <c r="D103" s="158">
+        <f>SUM(D101:D102)</f>
         <v>141026.91999999998</v>
       </c>
-      <c r="E94" s="147">
-        <f t="shared" ref="E94:F94" si="17">SUM(E92:E93)</f>
+      <c r="E103" s="147">
+        <f t="shared" ref="E103:F103" si="17">SUM(E101:E102)</f>
         <v>129617.84217199999</v>
       </c>
-      <c r="F94" s="147">
+      <c r="F103" s="147">
         <f t="shared" si="17"/>
         <v>11409.077827999999</v>
       </c>
-      <c r="G94" s="109">
-        <f>E94+F94</f>
+      <c r="G103" s="109">
+        <f>E103+F103</f>
         <v>141026.91999999998</v>
       </c>
-      <c r="H94" s="150" t="str">
-        <f>IF(D94=G94, "", "Error")</f>
+      <c r="H103" s="150" t="str">
+        <f>IF(D103=G103, "", "Error")</f>
         <v/>
       </c>
     </row>
-    <row r="95" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A95" s="7"/>
-      <c r="B95" s="7"/>
-      <c r="C95" s="7"/>
-      <c r="D95" s="190"/>
-      <c r="E95" s="12"/>
-      <c r="F95" s="7"/>
-      <c r="H95" s="150"/>
-    </row>
-    <row r="96" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A96" s="99" t="s">
+    <row r="104" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A104" s="7"/>
+      <c r="B104" s="7"/>
+      <c r="C104" s="7"/>
+      <c r="D104" s="190"/>
+      <c r="E104" s="12"/>
+      <c r="F104" s="7"/>
+      <c r="H104" s="150"/>
+    </row>
+    <row r="105" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A105" s="99" t="s">
         <v>134</v>
       </c>
-      <c r="B96" s="99"/>
-      <c r="C96" s="99"/>
-      <c r="D96" s="191"/>
-      <c r="E96" s="118">
-        <f>D96*91.91%</f>
-        <v>0</v>
-      </c>
-      <c r="F96" s="136">
-        <f>D96*8.09%</f>
-        <v>0</v>
-      </c>
-      <c r="G96" s="109">
-        <f>E96+F96</f>
-        <v>0</v>
-      </c>
-      <c r="H96" s="150" t="str">
-        <f>IF(D96=G96, "", "Error")</f>
+      <c r="B105" s="99"/>
+      <c r="C105" s="99"/>
+      <c r="D105" s="191"/>
+      <c r="E105" s="118">
+        <f>D105*91.91%</f>
+        <v>0</v>
+      </c>
+      <c r="F105" s="136">
+        <f>D105*8.09%</f>
+        <v>0</v>
+      </c>
+      <c r="G105" s="109">
+        <f>E105+F105</f>
+        <v>0</v>
+      </c>
+      <c r="H105" s="150" t="str">
+        <f>IF(D105=G105, "", "Error")</f>
         <v/>
       </c>
     </row>
-    <row r="97" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A97" s="1"/>
-      <c r="D97" s="188"/>
-      <c r="E97" s="2"/>
-      <c r="F97" s="10"/>
-      <c r="G97" s="157">
-        <f>SUM(G27:G96)</f>
-        <v>8586911.8399999999</v>
-      </c>
-      <c r="H97" s="150"/>
-    </row>
-    <row r="98" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A98" s="4" t="s">
+    <row r="106" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A106" s="1"/>
+      <c r="D106" s="188"/>
+      <c r="E106" s="2"/>
+      <c r="F106" s="10"/>
+      <c r="G106" s="157">
+        <f>SUM(G27:G105)</f>
+        <v>8796045.7599999998</v>
+      </c>
+      <c r="H106" s="150"/>
+    </row>
+    <row r="107" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A107" s="4" t="s">
         <v>104</v>
       </c>
-      <c r="B98" s="60"/>
-      <c r="C98" s="5"/>
-      <c r="D98" s="192">
-        <f>SUM(D96+D94+D90+D83+D76+D55+D35+D30+D48)</f>
-        <v>5277698.88</v>
-      </c>
-      <c r="E98" s="148">
-        <f>SUM(E96+E94+E90+E83+E76+E55+E35+E30+E48)</f>
-        <v>4946534.4161080001</v>
-      </c>
-      <c r="F98" s="148">
-        <f>SUM(F96+F94+F90+F83+F76+F55+F35+F30+F48)</f>
-        <v>331164.46389200003</v>
-      </c>
-      <c r="G98" s="109">
-        <f>E98+F98</f>
-        <v>5277698.88</v>
-      </c>
-      <c r="H98" s="150" t="str">
-        <f>IF(D98=G98, "", "Error")</f>
+      <c r="B107" s="60"/>
+      <c r="C107" s="5"/>
+      <c r="D107" s="192">
+        <f>SUM(D105+D103+D99+D92+D85+D55+D35+D30+D48)</f>
+        <v>5848392.3399999999</v>
+      </c>
+      <c r="E107" s="148">
+        <f>SUM(E105+E103+E99+E92+E85+E55+E35+E30+E48)</f>
+        <v>5317471.9837839995</v>
+      </c>
+      <c r="F107" s="148">
+        <f>SUM(F105+F103+F99+F92+F85+F55+F35+F30+F48)</f>
+        <v>333498.29621600005</v>
+      </c>
+      <c r="G107" s="109">
+        <f>E107+F107</f>
+        <v>5650970.2799999993</v>
+      </c>
+      <c r="H107" s="150" t="str">
+        <f>IF(D107=G107, "", "Error")</f>
+        <v>Error</v>
+      </c>
+      <c r="I107" s="181">
+        <f>D107-G107</f>
+        <v>197422.06000000052</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D108" s="188"/>
+      <c r="E108" s="109"/>
+    </row>
+    <row r="109" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A109" s="142" t="s">
+        <v>121</v>
+      </c>
+      <c r="B109" s="141"/>
+      <c r="C109" s="141"/>
+      <c r="E109" s="109"/>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A110" s="1"/>
+      <c r="C110" s="139"/>
+      <c r="E110" s="109"/>
+    </row>
+    <row r="111" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A111" s="1"/>
+      <c r="C111" s="139"/>
+      <c r="E111" s="109"/>
+    </row>
+    <row r="112" spans="1:10" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A112" s="143" t="s">
+        <v>30</v>
+      </c>
+      <c r="B112" s="144"/>
+      <c r="C112" s="140">
+        <f>SUM(C110:C111)</f>
+        <v>0</v>
+      </c>
+      <c r="E112" s="109"/>
+    </row>
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E113" s="109"/>
+    </row>
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="E114" s="137"/>
+    </row>
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A115" s="225" t="s">
+        <v>114</v>
+      </c>
+      <c r="B115" s="226"/>
+      <c r="C115" s="226"/>
+      <c r="D115" s="226"/>
+      <c r="E115" s="172" t="s">
+        <v>22</v>
+      </c>
+      <c r="F115" s="173" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="116" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A116" s="222"/>
+      <c r="B116" s="223"/>
+      <c r="C116" s="224"/>
+      <c r="D116" s="167"/>
+      <c r="E116" s="149"/>
+      <c r="F116" s="134"/>
+    </row>
+    <row r="117" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A117" s="219"/>
+      <c r="B117" s="220"/>
+      <c r="C117" s="221"/>
+      <c r="D117" s="182"/>
+      <c r="E117" s="149"/>
+      <c r="F117" s="134"/>
+    </row>
+    <row r="118" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A118" s="174"/>
+      <c r="B118" s="175"/>
+      <c r="C118" s="176"/>
+      <c r="D118" s="182"/>
+      <c r="E118" s="149"/>
+      <c r="F118" s="134"/>
+    </row>
+    <row r="119" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A119" s="219"/>
+      <c r="B119" s="220"/>
+      <c r="C119" s="221"/>
+      <c r="D119" s="113"/>
+      <c r="E119" s="149">
+        <f>D119*91.91%</f>
+        <v>0</v>
+      </c>
+      <c r="F119" s="134">
+        <f>D119*8.09%</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A120" s="213" t="s">
+        <v>30</v>
+      </c>
+      <c r="B120" s="214"/>
+      <c r="C120" s="215"/>
+      <c r="D120" s="171">
+        <f>SUM(D116:D119)</f>
+        <v>0</v>
+      </c>
+      <c r="E120" s="171">
+        <f>SUM(E116:E119)</f>
+        <v>0</v>
+      </c>
+      <c r="F120" s="171">
+        <f>SUM(F116:F119)</f>
+        <v>0</v>
+      </c>
+      <c r="H120" s="109">
+        <f>E120+F120</f>
+        <v>0</v>
+      </c>
+      <c r="I120" s="150" t="str">
+        <f>IF(D120=H120, "", "Error")</f>
         <v/>
       </c>
-      <c r="I98" s="181">
-        <f>D98-G98</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="99" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="D99" s="188"/>
-      <c r="E99" s="109"/>
-    </row>
-    <row r="100" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A100" s="142" t="s">
-        <v>121</v>
-      </c>
-      <c r="B100" s="141"/>
-      <c r="C100" s="141"/>
-      <c r="E100" s="109"/>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A101" s="1"/>
-      <c r="C101" s="139"/>
-      <c r="E101" s="109"/>
-    </row>
-    <row r="102" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A102" s="1"/>
-      <c r="C102" s="139"/>
-      <c r="E102" s="109"/>
-    </row>
-    <row r="103" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A103" s="143" t="s">
-        <v>30</v>
-      </c>
-      <c r="B103" s="144"/>
-      <c r="C103" s="140">
-        <f>SUM(C101:C102)</f>
-        <v>0</v>
-      </c>
-      <c r="E103" s="109"/>
-    </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E104" s="109"/>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="E105" s="137"/>
-    </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A106" s="224" t="s">
-        <v>114</v>
-      </c>
-      <c r="B106" s="225"/>
-      <c r="C106" s="225"/>
-      <c r="D106" s="225"/>
-      <c r="E106" s="172" t="s">
-        <v>22</v>
-      </c>
-      <c r="F106" s="173" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="107" spans="1:9" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A107" s="221"/>
-      <c r="B107" s="222"/>
-      <c r="C107" s="223"/>
-      <c r="D107" s="167"/>
-      <c r="E107" s="149"/>
-      <c r="F107" s="134"/>
-    </row>
-    <row r="108" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A108" s="218"/>
-      <c r="B108" s="219"/>
-      <c r="C108" s="220"/>
-      <c r="D108" s="182"/>
-      <c r="E108" s="149"/>
-      <c r="F108" s="134"/>
-    </row>
-    <row r="109" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="174"/>
-      <c r="B109" s="175"/>
-      <c r="C109" s="176"/>
-      <c r="D109" s="182"/>
-      <c r="E109" s="149"/>
-      <c r="F109" s="134"/>
-    </row>
-    <row r="110" spans="1:9" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A110" s="218"/>
-      <c r="B110" s="219"/>
-      <c r="C110" s="220"/>
-      <c r="D110" s="113"/>
-      <c r="E110" s="149">
-        <f>D110*91.91%</f>
-        <v>0</v>
-      </c>
-      <c r="F110" s="134">
-        <f>D110*8.09%</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A111" s="212" t="s">
-        <v>30</v>
-      </c>
-      <c r="B111" s="213"/>
-      <c r="C111" s="214"/>
-      <c r="D111" s="171">
-        <f>SUM(D107:D110)</f>
-        <v>0</v>
-      </c>
-      <c r="E111" s="171">
-        <f>SUM(E107:E110)</f>
-        <v>0</v>
-      </c>
-      <c r="F111" s="171">
-        <f>SUM(F107:F110)</f>
-        <v>0</v>
-      </c>
-      <c r="H111" s="109">
-        <f>E111+F111</f>
-        <v>0</v>
-      </c>
-      <c r="I111" s="150" t="str">
-        <f>IF(D111=H111, "", "Error")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="113" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="E113" s="109"/>
-    </row>
-    <row r="114" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A114" s="102" t="s">
+    </row>
+    <row r="122" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="E122" s="109"/>
+    </row>
+    <row r="123" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A123" s="102" t="s">
         <v>105</v>
       </c>
-      <c r="B114" s="103">
-        <f>D98</f>
-        <v>5277698.88</v>
-      </c>
-    </row>
-    <row r="115" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A115" s="104" t="s">
+      <c r="B123" s="103">
+        <f>D107</f>
+        <v>5848392.3399999999</v>
+      </c>
+    </row>
+    <row r="124" spans="1:9" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A124" s="104" t="s">
         <v>107</v>
       </c>
-      <c r="B115" s="105">
-        <f>D98-D96</f>
-        <v>5277698.88</v>
-      </c>
-    </row>
-    <row r="116" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="D116" s="202"/>
-      <c r="E116" s="202"/>
-    </row>
-    <row r="117" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A117" s="74" t="s">
+      <c r="B124" s="105">
+        <f>D107-D105</f>
+        <v>5848392.3399999999</v>
+      </c>
+    </row>
+    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="D125" s="233"/>
+      <c r="E125" s="233"/>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A126" s="74" t="s">
         <v>91</v>
       </c>
-      <c r="B117" s="75"/>
-      <c r="C117" s="76"/>
-      <c r="D117" s="202"/>
-      <c r="E117" s="202"/>
-    </row>
-    <row r="118" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A118" s="77" t="s">
+      <c r="B126" s="75"/>
+      <c r="C126" s="76"/>
+      <c r="D126" s="233"/>
+      <c r="E126" s="233"/>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A127" s="77" t="s">
         <v>92</v>
       </c>
-      <c r="B118" s="78">
+      <c r="B127" s="78">
         <v>4452323.820828055</v>
       </c>
-      <c r="C118" s="78"/>
-      <c r="D118" s="202"/>
-      <c r="E118" s="202"/>
-    </row>
-    <row r="119" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A119" s="79" t="s">
+      <c r="C127" s="78"/>
+      <c r="D127" s="233"/>
+      <c r="E127" s="233"/>
+    </row>
+    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A128" s="79" t="s">
         <v>93</v>
       </c>
-      <c r="B119" s="92">
+      <c r="B128" s="92">
         <f>PRORRATEO!G52</f>
         <v>6849105.1357215978</v>
       </c>
-      <c r="C119" s="78" t="s">
+      <c r="C128" s="78" t="s">
         <v>94</v>
       </c>
-      <c r="D119" s="202"/>
-      <c r="E119" s="202"/>
-    </row>
-    <row r="120" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A120" s="79" t="s">
+      <c r="D128" s="233"/>
+      <c r="E128" s="233"/>
+    </row>
+    <row r="129" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A129" s="79" t="s">
         <v>116</v>
       </c>
-      <c r="B120" s="178">
-        <f>-B115</f>
-        <v>-5277698.88</v>
-      </c>
-      <c r="C120" s="76"/>
-      <c r="D120" s="202"/>
-      <c r="E120" s="202"/>
-      <c r="G120" s="113"/>
-    </row>
-    <row r="121" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A121" s="79" t="s">
+      <c r="B129" s="178">
+        <f>-B124</f>
+        <v>-5848392.3399999999</v>
+      </c>
+      <c r="C129" s="76"/>
+      <c r="D129" s="233"/>
+      <c r="E129" s="233"/>
+      <c r="G129" s="113"/>
+    </row>
+    <row r="130" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A130" s="79" t="s">
         <v>115</v>
       </c>
-      <c r="B121" s="178">
-        <f>-D111</f>
-        <v>0</v>
-      </c>
-      <c r="C121" s="76"/>
-      <c r="D121" s="202"/>
-      <c r="E121" s="202"/>
-      <c r="G121" s="125"/>
-    </row>
-    <row r="122" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A122" s="79" t="s">
+      <c r="B130" s="178">
+        <f>-D120</f>
+        <v>0</v>
+      </c>
+      <c r="C130" s="76"/>
+      <c r="D130" s="233"/>
+      <c r="E130" s="233"/>
+      <c r="G130" s="125"/>
+    </row>
+    <row r="131" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A131" s="79" t="s">
         <v>106</v>
       </c>
-      <c r="B122" s="178">
-        <f>-B129</f>
-        <v>0</v>
-      </c>
-      <c r="C122" s="80"/>
-    </row>
-    <row r="123" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A123" s="79" t="s">
+      <c r="B131" s="178">
+        <f>-B138</f>
+        <v>0</v>
+      </c>
+      <c r="C131" s="80"/>
+    </row>
+    <row r="132" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A132" s="79" t="s">
         <v>121</v>
       </c>
-      <c r="B123" s="93">
-        <f>-C103</f>
-        <v>0</v>
-      </c>
-      <c r="C123" s="80"/>
-    </row>
-    <row r="124" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A124" s="79"/>
-      <c r="B124" s="75"/>
-      <c r="C124" s="80"/>
-    </row>
-    <row r="125" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A125" s="77" t="s">
+      <c r="B132" s="93">
+        <f>-C112</f>
+        <v>0</v>
+      </c>
+      <c r="C132" s="80"/>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A133" s="79"/>
+      <c r="B133" s="75"/>
+      <c r="C133" s="80"/>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A134" s="77" t="s">
         <v>95</v>
       </c>
-      <c r="B125" s="81">
-        <f>SUM(B118:B124)</f>
-        <v>6023730.076549652</v>
-      </c>
-      <c r="C125" s="154"/>
-    </row>
-    <row r="126" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A126" s="80"/>
-      <c r="C126" s="76"/>
-      <c r="D126" s="83"/>
-    </row>
-    <row r="127" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="C127" s="76"/>
-      <c r="D127" s="109"/>
-      <c r="E127" s="181"/>
-    </row>
-    <row r="128" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A128" s="74" t="s">
+      <c r="B134" s="81">
+        <f>SUM(B127:B133)</f>
+        <v>5453036.6165496521</v>
+      </c>
+      <c r="C134" s="154"/>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A135" s="80"/>
+      <c r="C135" s="76"/>
+      <c r="D135" s="83"/>
+    </row>
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C136" s="76"/>
+      <c r="D136" s="109"/>
+      <c r="E136" s="181"/>
+    </row>
+    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A137" s="74" t="s">
         <v>96</v>
       </c>
-      <c r="B128" s="11">
+      <c r="B137" s="11">
         <v>-310694.54000000004</v>
       </c>
-      <c r="C128" s="82"/>
-    </row>
-    <row r="129" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A129" s="77" t="s">
-        <v>164</v>
-      </c>
-      <c r="B129" s="93"/>
-      <c r="C129" s="82"/>
-      <c r="D129" s="181"/>
-      <c r="E129" s="109"/>
-    </row>
-    <row r="130" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A130" s="77"/>
-      <c r="B130" s="178"/>
-      <c r="C130" s="82"/>
-      <c r="E130" s="109"/>
-    </row>
-    <row r="131" spans="1:14" hidden="1" x14ac:dyDescent="0.3">
-      <c r="A131" s="77"/>
-      <c r="B131" s="178"/>
-      <c r="C131" s="82"/>
-      <c r="E131" s="109"/>
-    </row>
-    <row r="132" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A132" s="77"/>
-      <c r="B132" s="178"/>
-      <c r="C132" s="82"/>
-      <c r="E132" s="109"/>
-    </row>
-    <row r="133" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A133" s="100" t="s">
+      <c r="C137" s="82"/>
+    </row>
+    <row r="138" spans="1:7" ht="14.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A138" s="77" t="s">
+        <v>156</v>
+      </c>
+      <c r="B138" s="93"/>
+      <c r="C138" s="82"/>
+      <c r="D138" s="181"/>
+      <c r="E138" s="109"/>
+    </row>
+    <row r="139" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A139" s="77"/>
+      <c r="B139" s="178"/>
+      <c r="C139" s="82"/>
+      <c r="E139" s="109"/>
+    </row>
+    <row r="140" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
+      <c r="A140" s="77"/>
+      <c r="B140" s="178"/>
+      <c r="C140" s="82"/>
+      <c r="E140" s="109"/>
+    </row>
+    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A141" s="77"/>
+      <c r="B141" s="178"/>
+      <c r="C141" s="82"/>
+      <c r="E141" s="109"/>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A142" s="100" t="s">
         <v>30</v>
       </c>
-      <c r="B133" s="101">
-        <f>SUM(B128:B132)</f>
+      <c r="B142" s="101">
+        <f>SUM(B137:B141)</f>
         <v>-310694.54000000004</v>
       </c>
-      <c r="C133" s="82"/>
-    </row>
-    <row r="134" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="C134" s="83"/>
-      <c r="D134" s="181"/>
-    </row>
-    <row r="135" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B135" s="80"/>
-      <c r="C135" s="76"/>
-    </row>
-    <row r="137" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="N137" s="12"/>
-    </row>
-    <row r="140" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B140" s="201" t="s">
-        <v>163</v>
-      </c>
-      <c r="C140" s="201"/>
-      <c r="D140" s="201"/>
-      <c r="E140" s="201"/>
-    </row>
-    <row r="141" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B141" s="201"/>
-      <c r="C141" s="201"/>
-      <c r="D141" s="201"/>
-      <c r="E141" s="201"/>
-    </row>
-    <row r="142" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B142" s="201"/>
-      <c r="C142" s="201"/>
-      <c r="D142" s="201"/>
-      <c r="E142" s="201"/>
-    </row>
-    <row r="143" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B143" s="201"/>
-      <c r="C143" s="201"/>
-      <c r="D143" s="201"/>
-      <c r="E143" s="201"/>
-    </row>
-    <row r="144" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="B144" s="201"/>
-      <c r="C144" s="201"/>
-      <c r="D144" s="201"/>
-      <c r="E144" s="201"/>
+      <c r="C142" s="82"/>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="C143" s="83"/>
+      <c r="D143" s="181"/>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B144" s="80"/>
+      <c r="C144" s="76"/>
+    </row>
+    <row r="146" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="N146" s="12"/>
+    </row>
+    <row r="149" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B149" s="232" t="s">
+        <v>155</v>
+      </c>
+      <c r="C149" s="232"/>
+      <c r="D149" s="232"/>
+      <c r="E149" s="232"/>
+    </row>
+    <row r="150" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B150" s="232"/>
+      <c r="C150" s="232"/>
+      <c r="D150" s="232"/>
+      <c r="E150" s="232"/>
+    </row>
+    <row r="151" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B151" s="232"/>
+      <c r="C151" s="232"/>
+      <c r="D151" s="232"/>
+      <c r="E151" s="232"/>
+    </row>
+    <row r="152" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B152" s="232"/>
+      <c r="C152" s="232"/>
+      <c r="D152" s="232"/>
+      <c r="E152" s="232"/>
+    </row>
+    <row r="153" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B153" s="232"/>
+      <c r="C153" s="232"/>
+      <c r="D153" s="232"/>
+      <c r="E153" s="232"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="B140:E144"/>
-    <mergeCell ref="D116:E121"/>
+  <mergeCells count="17">
+    <mergeCell ref="B149:E153"/>
+    <mergeCell ref="D125:E130"/>
     <mergeCell ref="B14:D17"/>
-    <mergeCell ref="A111:C111"/>
-    <mergeCell ref="A66:C66"/>
-    <mergeCell ref="A108:C108"/>
-    <mergeCell ref="A110:C110"/>
-    <mergeCell ref="A107:C107"/>
-    <mergeCell ref="A106:D106"/>
+    <mergeCell ref="A120:C120"/>
+    <mergeCell ref="A68:C68"/>
+    <mergeCell ref="A117:C117"/>
+    <mergeCell ref="A119:C119"/>
+    <mergeCell ref="A116:C116"/>
+    <mergeCell ref="A115:D115"/>
+    <mergeCell ref="A77:C77"/>
+    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A74:C74"/>
     <mergeCell ref="A69:C69"/>
-    <mergeCell ref="A65:C65"/>
-    <mergeCell ref="A67:C67"/>
+    <mergeCell ref="A70:C70"/>
+    <mergeCell ref="A71:C71"/>
+    <mergeCell ref="A78:B78"/>
+    <mergeCell ref="A75:C75"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -3996,15 +4176,15 @@
       <c r="K1" s="8" t="s">
         <v>125</v>
       </c>
-      <c r="L1" s="228">
-        <f>RESUMEN!D98</f>
-        <v>5277698.88</v>
-      </c>
-      <c r="M1" s="229"/>
+      <c r="L1" s="240">
+        <f>RESUMEN!D107</f>
+        <v>5848392.3399999999</v>
+      </c>
+      <c r="M1" s="241"/>
       <c r="N1" s="152"/>
       <c r="O1" s="135">
         <f>L1*8.09%</f>
-        <v>426965.83939199999</v>
+        <v>473134.940306</v>
       </c>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
@@ -4029,7 +4209,7 @@
       <c r="N2" s="153"/>
       <c r="O2" s="135">
         <f>O1-K7-553-50-86-8</f>
-        <v>95338.539740999986</v>
+        <v>141507.640655</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
@@ -4076,64 +4256,64 @@
       <c r="N4" s="124"/>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A5" s="226" t="s">
+      <c r="A5" s="234" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="239" t="s">
+      <c r="B5" s="236" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="226" t="s">
+      <c r="C5" s="234" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="237" t="s">
+      <c r="D5" s="238" t="s">
         <v>23</v>
       </c>
-      <c r="E5" s="226" t="s">
+      <c r="E5" s="234" t="s">
         <v>98</v>
       </c>
-      <c r="F5" s="226" t="s">
+      <c r="F5" s="234" t="s">
         <v>24</v>
       </c>
-      <c r="G5" s="226" t="s">
+      <c r="G5" s="234" t="s">
         <v>25</v>
       </c>
-      <c r="H5" s="232" t="s">
+      <c r="H5" s="244" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="237" t="s">
+      <c r="I5" s="238" t="s">
         <v>109</v>
       </c>
-      <c r="J5" s="230" t="s">
+      <c r="J5" s="242" t="s">
         <v>27</v>
       </c>
-      <c r="K5" s="230" t="s">
+      <c r="K5" s="242" t="s">
         <v>70</v>
       </c>
-      <c r="L5" s="235" t="s">
+      <c r="L5" s="247" t="s">
         <v>124</v>
       </c>
-      <c r="M5" s="230" t="s">
+      <c r="M5" s="242" t="s">
         <v>68</v>
       </c>
-      <c r="N5" s="230" t="s">
+      <c r="N5" s="242" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A6" s="227"/>
-      <c r="B6" s="240"/>
-      <c r="C6" s="227"/>
-      <c r="D6" s="241"/>
-      <c r="E6" s="227"/>
-      <c r="F6" s="227"/>
-      <c r="G6" s="227"/>
-      <c r="H6" s="233"/>
-      <c r="I6" s="238"/>
-      <c r="J6" s="231"/>
-      <c r="K6" s="234"/>
-      <c r="L6" s="236"/>
-      <c r="M6" s="234"/>
-      <c r="N6" s="231"/>
+      <c r="A6" s="235"/>
+      <c r="B6" s="237"/>
+      <c r="C6" s="235"/>
+      <c r="D6" s="239"/>
+      <c r="E6" s="235"/>
+      <c r="F6" s="235"/>
+      <c r="G6" s="235"/>
+      <c r="H6" s="245"/>
+      <c r="I6" s="249"/>
+      <c r="J6" s="243"/>
+      <c r="K6" s="246"/>
+      <c r="L6" s="248"/>
+      <c r="M6" s="246"/>
+      <c r="N6" s="243"/>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="7" t="s">
@@ -4579,7 +4759,7 @@
         <v>32</v>
       </c>
       <c r="D16" s="133" t="s">
-        <v>155</v>
+        <v>148</v>
       </c>
       <c r="E16" s="7">
         <v>2.84</v>
@@ -5911,7 +6091,7 @@
       </c>
       <c r="P43" s="109">
         <f>L1-K52</f>
-        <v>32595.47104900144</v>
+        <v>603288.9310490014</v>
       </c>
     </row>
     <row r="44" spans="1:17" x14ac:dyDescent="0.3">
@@ -6340,36 +6520,36 @@
     <row r="53" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
       <c r="K53" s="138">
         <f>K52-L1</f>
-        <v>-32595.47104900144</v>
+        <v>-603288.9310490014</v>
       </c>
     </row>
     <row r="54" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C54" s="202"/>
-      <c r="D54" s="202"/>
-      <c r="E54" s="202"/>
-      <c r="F54" s="202"/>
-      <c r="G54" s="202"/>
-      <c r="H54" s="202"/>
-      <c r="I54" s="202"/>
-      <c r="J54" s="202"/>
-      <c r="K54" s="202"/>
-      <c r="L54" s="202"/>
-      <c r="M54" s="202"/>
-      <c r="N54" s="202"/>
+      <c r="C54" s="233"/>
+      <c r="D54" s="233"/>
+      <c r="E54" s="233"/>
+      <c r="F54" s="233"/>
+      <c r="G54" s="233"/>
+      <c r="H54" s="233"/>
+      <c r="I54" s="233"/>
+      <c r="J54" s="233"/>
+      <c r="K54" s="233"/>
+      <c r="L54" s="233"/>
+      <c r="M54" s="233"/>
+      <c r="N54" s="233"/>
     </row>
     <row r="55" spans="1:16" hidden="1" x14ac:dyDescent="0.3">
-      <c r="C55" s="202"/>
-      <c r="D55" s="202"/>
-      <c r="E55" s="202"/>
-      <c r="F55" s="202"/>
-      <c r="G55" s="202"/>
-      <c r="H55" s="202"/>
-      <c r="I55" s="202"/>
-      <c r="J55" s="202"/>
-      <c r="K55" s="202"/>
-      <c r="L55" s="202"/>
-      <c r="M55" s="202"/>
-      <c r="N55" s="202"/>
+      <c r="C55" s="233"/>
+      <c r="D55" s="233"/>
+      <c r="E55" s="233"/>
+      <c r="F55" s="233"/>
+      <c r="G55" s="233"/>
+      <c r="H55" s="233"/>
+      <c r="I55" s="233"/>
+      <c r="J55" s="233"/>
+      <c r="K55" s="233"/>
+      <c r="L55" s="233"/>
+      <c r="M55" s="233"/>
+      <c r="N55" s="233"/>
     </row>
     <row r="56" spans="1:16" x14ac:dyDescent="0.3">
       <c r="C56" s="169"/>
@@ -6386,112 +6566,107 @@
       <c r="N56" s="169"/>
     </row>
     <row r="57" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="C57" s="202" t="s">
+      <c r="C57" s="233" t="s">
         <v>130</v>
       </c>
-      <c r="D57" s="202"/>
-      <c r="E57" s="202"/>
-      <c r="F57" s="202"/>
-      <c r="G57" s="202"/>
-      <c r="H57" s="202"/>
-      <c r="I57" s="202"/>
-      <c r="J57" s="202"/>
-      <c r="K57" s="202"/>
-      <c r="L57" s="202"/>
-      <c r="M57" s="202"/>
-      <c r="N57" s="202"/>
+      <c r="D57" s="233"/>
+      <c r="E57" s="233"/>
+      <c r="F57" s="233"/>
+      <c r="G57" s="233"/>
+      <c r="H57" s="233"/>
+      <c r="I57" s="233"/>
+      <c r="J57" s="233"/>
+      <c r="K57" s="233"/>
+      <c r="L57" s="233"/>
+      <c r="M57" s="233"/>
+      <c r="N57" s="233"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="C58" s="202"/>
-      <c r="D58" s="202"/>
-      <c r="E58" s="202"/>
-      <c r="F58" s="202"/>
-      <c r="G58" s="202"/>
-      <c r="H58" s="202"/>
-      <c r="I58" s="202"/>
-      <c r="J58" s="202"/>
-      <c r="K58" s="202"/>
-      <c r="L58" s="202"/>
-      <c r="M58" s="202"/>
-      <c r="N58" s="202"/>
+      <c r="C58" s="233"/>
+      <c r="D58" s="233"/>
+      <c r="E58" s="233"/>
+      <c r="F58" s="233"/>
+      <c r="G58" s="233"/>
+      <c r="H58" s="233"/>
+      <c r="I58" s="233"/>
+      <c r="J58" s="233"/>
+      <c r="K58" s="233"/>
+      <c r="L58" s="233"/>
+      <c r="M58" s="233"/>
+      <c r="N58" s="233"/>
     </row>
     <row r="59" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="C59" s="202"/>
-      <c r="D59" s="202"/>
-      <c r="E59" s="202"/>
-      <c r="F59" s="202"/>
-      <c r="G59" s="202"/>
-      <c r="H59" s="202"/>
-      <c r="I59" s="202"/>
-      <c r="J59" s="202"/>
-      <c r="K59" s="202"/>
-      <c r="L59" s="202"/>
-      <c r="M59" s="202"/>
-      <c r="N59" s="202"/>
+      <c r="C59" s="233"/>
+      <c r="D59" s="233"/>
+      <c r="E59" s="233"/>
+      <c r="F59" s="233"/>
+      <c r="G59" s="233"/>
+      <c r="H59" s="233"/>
+      <c r="I59" s="233"/>
+      <c r="J59" s="233"/>
+      <c r="K59" s="233"/>
+      <c r="L59" s="233"/>
+      <c r="M59" s="233"/>
+      <c r="N59" s="233"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="C60" s="202"/>
-      <c r="D60" s="202"/>
-      <c r="E60" s="202"/>
-      <c r="F60" s="202"/>
-      <c r="G60" s="202"/>
-      <c r="H60" s="202"/>
-      <c r="I60" s="202"/>
-      <c r="J60" s="202"/>
-      <c r="K60" s="202"/>
-      <c r="L60" s="202"/>
-      <c r="M60" s="202"/>
-      <c r="N60" s="202"/>
+      <c r="C60" s="233"/>
+      <c r="D60" s="233"/>
+      <c r="E60" s="233"/>
+      <c r="F60" s="233"/>
+      <c r="G60" s="233"/>
+      <c r="H60" s="233"/>
+      <c r="I60" s="233"/>
+      <c r="J60" s="233"/>
+      <c r="K60" s="233"/>
+      <c r="L60" s="233"/>
+      <c r="M60" s="233"/>
+      <c r="N60" s="233"/>
     </row>
     <row r="61" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="C61" s="202"/>
-      <c r="D61" s="202"/>
-      <c r="E61" s="202"/>
-      <c r="F61" s="202"/>
-      <c r="G61" s="202"/>
-      <c r="H61" s="202"/>
-      <c r="I61" s="202"/>
-      <c r="J61" s="202"/>
-      <c r="K61" s="202"/>
-      <c r="L61" s="202"/>
-      <c r="M61" s="202"/>
-      <c r="N61" s="202"/>
+      <c r="C61" s="233"/>
+      <c r="D61" s="233"/>
+      <c r="E61" s="233"/>
+      <c r="F61" s="233"/>
+      <c r="G61" s="233"/>
+      <c r="H61" s="233"/>
+      <c r="I61" s="233"/>
+      <c r="J61" s="233"/>
+      <c r="K61" s="233"/>
+      <c r="L61" s="233"/>
+      <c r="M61" s="233"/>
+      <c r="N61" s="233"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="C62" s="202"/>
-      <c r="D62" s="202"/>
-      <c r="E62" s="202"/>
-      <c r="F62" s="202"/>
-      <c r="G62" s="202"/>
-      <c r="H62" s="202"/>
-      <c r="I62" s="202"/>
-      <c r="J62" s="202"/>
-      <c r="K62" s="202"/>
-      <c r="L62" s="202"/>
-      <c r="M62" s="202"/>
-      <c r="N62" s="202"/>
+      <c r="C62" s="233"/>
+      <c r="D62" s="233"/>
+      <c r="E62" s="233"/>
+      <c r="F62" s="233"/>
+      <c r="G62" s="233"/>
+      <c r="H62" s="233"/>
+      <c r="I62" s="233"/>
+      <c r="J62" s="233"/>
+      <c r="K62" s="233"/>
+      <c r="L62" s="233"/>
+      <c r="M62" s="233"/>
+      <c r="N62" s="233"/>
     </row>
     <row r="63" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="C63" s="202"/>
-      <c r="D63" s="202"/>
-      <c r="E63" s="202"/>
-      <c r="F63" s="202"/>
-      <c r="G63" s="202"/>
-      <c r="H63" s="202"/>
-      <c r="I63" s="202"/>
-      <c r="J63" s="202"/>
-      <c r="K63" s="202"/>
-      <c r="L63" s="202"/>
-      <c r="M63" s="202"/>
-      <c r="N63" s="202"/>
+      <c r="C63" s="233"/>
+      <c r="D63" s="233"/>
+      <c r="E63" s="233"/>
+      <c r="F63" s="233"/>
+      <c r="G63" s="233"/>
+      <c r="H63" s="233"/>
+      <c r="I63" s="233"/>
+      <c r="J63" s="233"/>
+      <c r="K63" s="233"/>
+      <c r="L63" s="233"/>
+      <c r="M63" s="233"/>
+      <c r="N63" s="233"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="C57:N63"/>
     <mergeCell ref="C54:N55"/>
@@ -6504,6 +6679,11 @@
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="I5:I6"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -6610,10 +6790,10 @@
       <c r="O4" s="49"/>
     </row>
     <row r="5" spans="1:15" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="242" t="s">
+      <c r="A5" s="250" t="s">
         <v>74</v>
       </c>
-      <c r="B5" s="242" t="s">
+      <c r="B5" s="250" t="s">
         <v>23</v>
       </c>
       <c r="C5" s="55" t="s">
@@ -6625,7 +6805,7 @@
       <c r="E5" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="F5" s="242" t="s">
+      <c r="F5" s="250" t="s">
         <v>76</v>
       </c>
       <c r="G5" s="37" t="s">
@@ -6647,16 +6827,16 @@
         <v>30</v>
       </c>
       <c r="M5" s="41"/>
-      <c r="N5" s="242" t="s">
+      <c r="N5" s="250" t="s">
         <v>79</v>
       </c>
-      <c r="O5" s="242" t="s">
+      <c r="O5" s="250" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A6" s="243"/>
-      <c r="B6" s="243"/>
+      <c r="A6" s="251"/>
+      <c r="B6" s="251"/>
       <c r="C6" s="56" t="s">
         <v>81</v>
       </c>
@@ -6666,7 +6846,7 @@
       <c r="E6" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="F6" s="243"/>
+      <c r="F6" s="251"/>
       <c r="G6" s="44" t="s">
         <v>82</v>
       </c>
@@ -6686,8 +6866,8 @@
         <v>85</v>
       </c>
       <c r="M6" s="47"/>
-      <c r="N6" s="243"/>
-      <c r="O6" s="243"/>
+      <c r="N6" s="251"/>
+      <c r="O6" s="251"/>
     </row>
     <row r="7" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="15">

</xml_diff>